<commit_message>
feat: extract and verify data for papers 203, 207, 208, 225 into canonical coding sheet
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/Full text coding sheet.xlsx
+++ b/03_Coding_Sheets/Full text coding sheet.xlsx
@@ -2564,10 +2564,14 @@
       </c>
       <c r="E30" s="28" t="inlineStr">
         <is>
-          <t>1 = Include</t>
-        </is>
-      </c>
-      <c r="F30" s="28" t="n"/>
+          <t>0 = Exclude</t>
+        </is>
+      </c>
+      <c r="F30" s="28" t="inlineStr">
+        <is>
+          <t>2 = Non-employee samples</t>
+        </is>
+      </c>
       <c r="G30" s="28" t="inlineStr">
         <is>
           <t>Extant management literature suggests that boundary spanning, defined as linking an organization's internal networks with external sources of information, is crucial to an organization’s growth and sustainability in that it enables firms to build connections, share knowledge, and exchange resources. A boundary spanner is a gatekeeper with access to external partners, critical resources, and information, and therefore, plays an important role in creating opportunities for an organization. This dissertation extends the research on individual boundary spanning by examining an overlooked source–skilled digital freelancers–and identifying how and when they are likely to serve as boundary spanners with a primary focus on their boundary spanning behaviors within contracted positions and the facilitating role of human capital and strategic orientation.</t>
@@ -18332,7 +18336,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1172" t="inlineStr">
+      <c r="Q1172" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -18427,7 +18431,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1173" t="inlineStr">
+      <c r="Q1173" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -18522,7 +18526,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1174" t="inlineStr">
+      <c r="Q1174" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -18617,7 +18621,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1175" t="inlineStr">
+      <c r="Q1175" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -18712,7 +18716,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1176" t="inlineStr">
+      <c r="Q1176" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -18807,7 +18811,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1177" t="inlineStr">
+      <c r="Q1177" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -18902,7 +18906,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1178" t="inlineStr">
+      <c r="Q1178" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -18997,7 +19001,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1179" t="inlineStr">
+      <c r="Q1179" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -19092,7 +19096,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1180" t="inlineStr">
+      <c r="Q1180" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -19187,7 +19191,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1181" t="inlineStr">
+      <c r="Q1181" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -19282,7 +19286,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1182" t="inlineStr">
+      <c r="Q1182" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -19377,7 +19381,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1183" t="inlineStr">
+      <c r="Q1183" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -19472,7 +19476,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1184" t="inlineStr">
+      <c r="Q1184" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -19567,7 +19571,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1185" t="inlineStr">
+      <c r="Q1185" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -19662,7 +19666,7 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1186" t="inlineStr">
+      <c r="Q1186" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
@@ -19757,12 +19761,12 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1187" t="inlineStr">
+      <c r="Q1187" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
       </c>
-      <c r="V1187" t="n">
+      <c r="V1187" s="0" t="n">
         <v>1461</v>
       </c>
       <c r="AA1187" s="0" t="n">
@@ -19851,12 +19855,12 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1188" t="inlineStr">
+      <c r="Q1188" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
       </c>
-      <c r="V1188" t="n">
+      <c r="V1188" s="0" t="n">
         <v>1461</v>
       </c>
       <c r="AA1188" s="0" t="n">
@@ -19945,12 +19949,12 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1189" t="inlineStr">
+      <c r="Q1189" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
       </c>
-      <c r="V1189" t="n">
+      <c r="V1189" s="0" t="n">
         <v>1461</v>
       </c>
       <c r="AA1189" s="0" t="n">
@@ -20039,12 +20043,12 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1190" t="inlineStr">
+      <c r="Q1190" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
       </c>
-      <c r="V1190" t="n">
+      <c r="V1190" s="0" t="n">
         <v>1461</v>
       </c>
       <c r="AA1190" s="0" t="n">
@@ -20133,12 +20137,12 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1191" t="inlineStr">
+      <c r="Q1191" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
       </c>
-      <c r="V1191" t="n">
+      <c r="V1191" s="0" t="n">
         <v>1461</v>
       </c>
       <c r="AA1191" s="0" t="n">
@@ -20227,12 +20231,12 @@
           <t>1 = include</t>
         </is>
       </c>
-      <c r="Q1192" t="inlineStr">
+      <c r="Q1192" s="0" t="inlineStr">
         <is>
           <t>2 = Longitudinal design</t>
         </is>
       </c>
-      <c r="V1192" t="n">
+      <c r="V1192" s="0" t="n">
         <v>1461</v>
       </c>
       <c r="AA1192" s="0" t="n">

</xml_diff>